<commit_message>
chore: update news radar report 2026-10-24
</commit_message>
<xml_diff>
--- a/docs/data/rxbenefits_intel_hub_report_2026-10-23.xlsx
+++ b/docs/data/rxbenefits_intel_hub_report_2026-10-23.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -477,27 +477,27 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>GLP-1 Compounder Recalls Copycat Zepbound Amid Safety Concerns</t>
+          <t>KFF Survey Shows Employer Health Insurance Premiums Surge Nearly 10%</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>A compounder has issued a recall for copycat Zepbound products, highlighting ongoing safety and quality risks associated with compounded GLP-1 medications. This development underscores the clinical and financial risks self-funded employers face when plan members turn to compounded alternatives amid high brand-name drug costs. The incident reinforces the importance of PBM-guided formulary management and safety education for employers navigating obesity drug coverage.</t>
+          <t>A new KFF report reveals that workers are paying nearly 10% more for family health insurance premiums on employer-sponsored plans. This rising cost burden underscores the ongoing pressure on self-funded employers to manage healthcare spending and reevaluate benefit plan designs.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BioPharma Dive</t>
+          <t>ABC News - Breaking News, Latest News and Videos</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 15:56:47 GMT</t>
+          <t>Fri, 23 Oct 2026 18:44:10 GMT</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxNMWtyNDBobVJtblN0ejdHbVFzejhSZllfNDNwUjZuSVBfSE1NeHczLVZTVzM1b2d0ME1FeGJTQk1ZV2ZOSFBtbmg0d3pReXBHRWtTTlFkc1M0YXlQeFFFdkNfbWVWM2NjbWt6MnVLNXVqb1Qyb3ZfaXhpcGo4STlVUDNYVlZYS0tXbkktNDlJNUhka1FhcUQ3UDgtdWtKOVkt?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxOaW02aTFDd3k5ZjJOSGtoN2FaVzdQT0tFSktQQU1LWXlteVlaZHJ6Z25HM184TEZBM25qcTFwWjFRNXlBb01adGQ1Y0t3Q216dUs5VnNqa09ZcjNBTWVCbGJla013TmxjZE5PdktBeDBSZVZxUTRQek1wQ1ZGSEhUZ1ZiU1ExeUJBYzNacUVXeF80b0NvNjFpeExuT3Q4eXJnczhldTIyOTDSAa4BQVVfeXFMTXJTbkRqa2o1d0Rzc3dMcEF0MU5JRlZrc2c5R1Z4dy1Pa3FsektzZ0ZOZVNmQlN0bHQteGZlcFdRTVQycnlfX181b1RWQk9nWGV3aU1FV1o5SjhxREJxNzFPZDVzc3pHNmFzNkRHX01LR2tFSHdlci1GMThKNFBzaC1qclIzZnNZSTgwYWRQTXl3a2RHYnhBSlB4bU96RThkTFB0dG5fSGxvcHVLdi1n?oc=5</t>
         </is>
       </c>
     </row>
@@ -507,27 +507,27 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Employer-Sponsored Family Health Coverage Premiurs Surpass $28,000 in 2026</t>
+          <t>Employer-Sponsored Health Insurance Costs Continue Escalating Nationwide</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Average annual premiums for employer-sponsored family health coverage have crossed the $28,000 threshold, underscoring escalating cost pressures on commercial health plans. This ongoing surge places intense pressure on self-funded employers to reevaluate their benefit strategies and seek aggressive cost-containment solutions for pharmacy and medical benefits.</t>
+          <t>A new nonpartisan survey reveals that the cost of employer-sponsored health plans has risen once again, putting additional financial strain on self-funded employers. Pharmacy benefits remain a major driver of these escalating healthcare costs, increasing the urgency for employers to adopt aggressive PBM cost-management and plan design strategies.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>KFF</t>
+          <t>InsuranceNewsNet</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 20:16:39 GMT</t>
+          <t>Fri, 23 Oct 2026 19:11:16 GMT</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxQdzZhd0FaYlAxRlRRRTF5VjRXcVdpa0FZMFEtYk11WHE2S3N5ZUZwRWpQZWRLTm1ybTg0MTNseGtKNTJ6OWtxVVBPZTJLeF9idzBlSWtfSHQxWXFXSzJfUjVUa1ZVcHFJQ0lTakktdVRXVDNHMlZ1X3NDOFNMbFAwb3VLQU5TdW5PNWZCUVhSdy0tUF8tVUhpcXBreE00VkxnbklNX0haLXhFeTda?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxOeXFaVnlGcHRnTWEyaXF0MmFCZnRvY2ZhYWF1OHhOc3Jld1RHc0Z2LXFVZFNDbzROMzZyc0xBRlpHYnFjZUxDMUJnbVplOFJaWjRPSEhjQ3JGejJrUEJsWmpNOHJrOTJ6Ym13R3pFckYyc2lKXzRXLVZRLXF5cGFCcVoyS3pMNHZjYkpHUnYzeWo0cDRVNnpDQngwdWZTczd2OGVuUkdERTQ0LUgyaERGSl9MRXJzVjdsUXpoTjdRY3FvZTNj?oc=5</t>
         </is>
       </c>
     </row>
@@ -537,27 +537,27 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>KFF Survey Shows Family Health Coverage Costs Reach Nearly $7,500 for Workers</t>
+          <t>Major Employers Sue UnitedHealth Over Alleged Bogus Health Claims</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>A new KFF report reveals that worker contributions for family health coverage have climbed to nearly $7,500 annually, underscoring escalating cost pressures on employer-sponsored plans. This relentless growth in healthcare and pharmacy expenses increases the urgency for self-funded employers to seek aggressive cost management and transparent PBM strategies.</t>
+          <t>Kraft Heinz and Aramark have filed a lawsuit against UnitedHealth, alleging the insurer manipulated health claims and costs. This high-profile litigation highlights growing friction between self-funded employers and health plan administrators regarding claims transparency and financial accountability.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>NewsNation</t>
+          <t>InsuranceNewsNet</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 22:47:51 GMT</t>
+          <t>Fri, 23 Oct 2026 15:11:03 GMT</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE5KaHptUjFNNWFSelhfV1ZUUWFGbzFXSVBKaWxzSnRaaTNpcWZZUFBKdHE1aTBXekF6cDRrNXNDRDQwYXkxYlRRRU94WldhVmhodlZOMmdnZE15cTZvcFg4NWRZejI2SHZrc0E2c1RpYkEzd9IBd0FVX3lxTFBVS2tqRVpjWVRsV3ZTVmdaREhjOFVBS0VWeFotTDJYcFlPQlVwYlZDMjhNSnZpeUJzLVNkYVJRSFM5QWxkdzVWdnN1OElyQzV3S2tfT2swZnRRUEQwMm5wSFpiY2xORUd6NURIV21DTWlHU1lycWEw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxPd29iOFNvTmVqMU5tSzhhc0REalpHbm5DMEFsblhMLWt2cjlWYVZXUHdFQkhkTDRqQm1XN0ZLdlhYYUR1N1lKc1lWQUhrUzRrNVFWR1VjZXBOTk1tWVVhUDh3NFNpTUxQMmI5SzlxSEJQbVlldEp6ekxXeTBqeWx1UUNIXy01Ykl2N29IdlVLQjZJRGFxZ1A0RHdUcFpWZWU1dGJR?oc=5</t>
         </is>
       </c>
     </row>
@@ -567,27 +567,27 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>KFF Survey Shows Employer Family Health Premiums Rise 5% to $28K</t>
+          <t>Integrating Copay Programs and Gross-to-Net Revenue Protection Strategies</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>The annual KFF employer health benefits survey reveals that average family coverage premiums increased by 5% to reach $28,000. This ongoing cost escalation puts mounting pressure on self-funded employers who bear the direct financial burden of healthcare and pharmacy benefit inflation. Plan sponsors will need to reevaluate their benefit strategies and cost-containment measures to manage these rising expenses.</t>
+          <t>This Drug Channels article examines the intersection of copay assistance programs and gross-to-net revenue optimization for pharmaceutical manufacturers. While focused on manufacturer revenue strategies rather than direct self-funded employer plan design, the underlying dynamics impact specialty drug pricing and rebate structures that affect PBM economics. However, it lacks direct, actionable relevance for self-funded employer health plan cost management today.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Fierce Healthcare</t>
+          <t>Drug Channels</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 09:00:22 GMT</t>
+          <t>Fri, 23 Oct 2026 10:00:00 GMT</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPTnlDN0w3TGM1cmNnbGJucFozMDJJRW45TTNXak9wMUZXV25MTUcwQmZHbzVOMS1xWVhFRFlwY0hISGJXcXY2bEFIb1g3WEh5SFgwVkpMazhfWk1BSmlSODR1MkE4X19JVVlCVk93b190eE4yWE94VTItWDFQTVpJbGF3RjNVdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigwFBVV95cUxPdUdsSWpoTkNhaUZPdzExRDlQZjltY1hHLXhJS0JRbFZoWEM0MG95dmhtX3RZVmpUc0xMZDlvY2dyRlYwSkhTUjhTT1h2cmpvczlkWDZVVmVMeERoVWZWenBNWGhfdXpEZE5zZW1nN01rUVFScnFweVMzdHVVTlNPVnN5aw?oc=5</t>
         </is>
       </c>
     </row>
@@ -597,27 +597,27 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Employer-Sponsored Health Insurance Costs Continue Upward Trend</t>
+          <t>Consumer Advocates Raise Concerns Over Employer-Sponsored Plan Benefit Designs</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>A new nonpartisan survey reveals that the cost of employer-sponsored health insurance plans has risen again, driven largely by escalating medical and pharmacy benefit expenditures. This ongoing inflation places mounting financial pressure on self-funded employers to adopt aggressive cost-containment and benefit-management strategies.</t>
+          <t>Consumer representatives are expressing growing concern that self-funded employer health plan designs may increasingly disadvantage sicker employees through shifting cost burdens. This trend highlights the ongoing tension between employer cost-management strategies and adequacy of coverage for high-utilization members. Self-funded plan sponsors must carefully balance affordability initiatives with equitable access to care.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>InsuranceNewsNet</t>
+          <t>BenefitsPRO</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 23:37:42 GMT</t>
+          <t>Fri, 23 Oct 2026 20:29:42 GMT</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixAFBVV95cUxPT0pzWUR6aXJYS1NmY3oyYXlxTE5XWnJzLU9Qa0U3Zmdyb0MwUkhUUlZzeVRTYm9IamlXbGxCaEs1bkNHQi1sa2MxaHVILXBkYmZuajNlOUhzcDZUWGJhMUoxM0xoQVZEamRqVnRaWmlCWGl3NjVuSmtkUDhHR0htaHJlTUx6TTI3a0RQX2VYUjFmejJLVmJvOXdnSGpxVmtVRjM3QlZwVXJZNDl3Z1N4TDdCQjRheldqOHVXV0xBa0x6c2NN?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPX2VRVC0tOEVnZGdWRjdpdEZJME1pWllvOHdrMnF4bmF0N2hMdDQzMzVjV3pzb3VYMmpDcDIxSU42M0U5QVlNa0FhWkVQVUNvYW5DWnFLUGFrLUxyMFNxNGxVaG1ucnBLN0R6V2hGY004OWdQZEw1UHpKMG1WZklqS2M1eHdHenF3TWRRZUpWcVRpako5TVJaN0dkejZ6MGhpaTdzcGZ3?oc=5</t>
         </is>
       </c>
     </row>
@@ -627,27 +627,27 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>The 340B Rebate Pilot Standoff Involves Court, Congress, and Drugmakers</t>
+          <t>Launch Prices for New Prescription Drugs Surge 35%</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Drug manufacturers, legal entities, and federal lawmakers remain locked in a contentious standoff regarding 340B drug rebate pilots. This ongoing battle significantly impacts drug pricing dynamics, supply chain economics, and pharmacy benefit management strategies for self-funded health plans.</t>
+          <t>A new report reveals that launch prices for newly approved prescription drugs surged by 35%, driving up gross drug costs for commercial plans. This steep inflation in launch pricing directly threatens the affordability of self-funded employer health plans, intensifying the need for aggressive PBM formulary management and cost containment strategies.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Pharmaceutical Commerce</t>
+          <t>BenefitsPRO</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 20:17:29 GMT</t>
+          <t>Fri, 23 Oct 2026 15:09:25 GMT</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxQdEN2bU45eTR2ak5TUFhrVVpwNkU3NmVPOVNWRUROdDhFdTRIVkdCLXR0VjlvczhYanRoRVVvOHhsMjFTN0xrb3R1VTZLX3pRdXBQNlFsei1nbFFROXJuX2Z3ZmZ1U0YtdVhzMFU5MHpTTU9MZXB1cHFzVFM5TmVqd3ZndW5wTHVW?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxOMUhiOXhxY09LQzRzeF9TVDU2bGJ1Wlo3aGZmZlhWWVdveFMybjByWkJaY3B3empCU3hPWFJMak14ZTdSRnhJOHhIM0pOTWoyaWNZMzgycWk2Nkg5U2p1R1Q3UXdQQkVuVXRHMXExcmdmYVp5Mnh5Q1QydXpDQ2g4TXpUUFF2enF0VG9jWlZmSEY5RnM?oc=5</t>
         </is>
       </c>
     </row>
@@ -657,27 +657,27 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>87% of Employers Consider Switching PBMs Upon Renewal</t>
+          <t>First PBM Integrates Instacart Health Fresh Funds Into Employer Benefits</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>A recent survey reveals that 87% of employers are looking to change their pharmacy benefit manager when their contracts come up for renewal, driven by mounting frustrations over cost and transparency. This trend highlights a major opportunity for alternative PBM models to capture market share from self-funded employers seeking better value.</t>
+          <t>A PBM has partnered with Instacart to incorporate Fresh Funds into employee benefits, allowing self-funded employers to offer targeted grocery stipends for nutrition and health. This development highlights an expanding trend where PBMs and health plan administrators move beyond traditional pharmacy to integrate food-as-medicine initiatives into corporate wellness. For self-funded employers, this offers a novel plan design option to address chronic conditions and total healthcare cost management.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>BenefitsPRO</t>
+          <t>Progressive Grocer</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 12:27:52 GMT</t>
+          <t>Fri, 23 Oct 2026 15:00:57 GMT</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQU0xVNC1wYm1maHNrcU00bWpnVnpRR1Jib1VTcEZtcE1Xc0p5cXRrQnBlN1V4RGg4NnBEeHA4cHNyZjVIdE1rQmdJTFpIbXVQb2lMRXFpUjBqdi1yNFdpQzg1Zm43eEJzUTN3Rzh4OFAtRzVjMVpJbWV3dldGbXNBS1BKN2dJNDFUWXdTN0VUM2pXUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPSVlrZXhTLWJ6eXJnN3VCdTJvMXdsOWVvaGR0dGluSXFvVGNQNi1ISUY0N3RpbldjNWNCbzF5OV9TY3h6S00xZFZsN1JkTVZzeWdDRzgtakxUcHJabkJEOERHdEstZndZZlVWTjgwbDVnemJTZGg1ZF9Bd3phMW1aQzAydFM2dkZxdGFOdEQ3YzVnOEVNNUE?oc=5</t>
         </is>
       </c>
     </row>
@@ -687,27 +687,27 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Strategic Management of GLP-1 Starter Doses Impacts Employer Plan Costs</t>
+          <t>House Oversight Committee Probes PBM Independent Pharmacy Audits</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>The article discusses how managing GLP-1 starter prescriptions effectively influences overall cost and adherence for employer-sponsored health plans. For self-funded employers and PBMs, optimizing initial prescribing and titration protocols is crucial to managing the massive financial impact of anti-obesity medications. Proper early management helps prevent waste from abandoned prescriptions and ensures long-term cost-effectiveness.</t>
+          <t>The House Oversight Committee has launched an inquiry into pharmacy benefit managers regarding their audit practices for independent pharmacies. This congressional scrutiny adds to the growing pressure on PBM transparency, contract practices, and regulatory oversight affecting self-funded health plans.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>BenefitsPRO</t>
+          <t>Fierce Healthcare</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 12:27:52 GMT</t>
+          <t>Fri, 23 Oct 2026 19:00:00 GMT</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTE1RSkJLSUlEVkMtMXhhSHFxa21QZUFXSWV0VFVyTGtmeG9SOGZUVXRZOFB5c29wZVljSjhsdnJHZGtDR2dRQndVUkdvYmkySVNoNFI4YVJaV0xTZWhZeEtmWUh3WG1VQ1hpSDBPczJCTVdFVmI3YkVxTUR4YUVKQk0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNc1NXdHBtMHZmX1k1ME41Z2d2VG13Z2xreGw3WjE3UlFJNHdVNkFtdjlERktkaFhmMzRvSjlUcjBlV1hjdWJwbnY1RGg1ZHpOcUhxVkZJVWZVRDRaa0ZFUC1jVzlLOUtIaU1PSmVsZlpGUktsaGpvcTl1cTR6NTU0TXRoU1VTRGtFYVc3RXhKS2ZzYzYxeXJlRllrQ00tbU9obFFvQ09sSmN2aHNMQURuXw?oc=5</t>
         </is>
       </c>
     </row>
@@ -717,27 +717,27 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>ERISA Fiduciary Litigation Expands Beyond Prescription Drugs to Voluntary Benefits</t>
+          <t>House Committee Launches Investigation Into Major PBMs</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Plaintiffs' attorneys are expanding ERISA breach of fiduciary duty lawsuits against self-funded employers from prescription drug benefits to include voluntary insurance products. This trend increases legal exposure for plan sponsors and highlights the growing scrutiny on all employer-sponsored health and welfare benefit arrangements. Self-funded employers must review their vendor contracts, fee disclosures, and administrative practices across all benefit lines to mitigate litigation risk.</t>
+          <t>The House Oversight Committee has initiated a formal probe into the three largest pharmacy benefit managers—Optum Rx, Express Scripts, and CVS Caremark—scrutinizing their business practices and pricing models. This congressional inquiry heightens regulatory pressure on traditional PBMs, signaling potential legislative shifts that could impact how self-funded employers contract for pharmacy benefits.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Buchanan Ingersoll &amp; Rooney PC</t>
+          <t>Modern Healthcare</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 14:27:04 GMT</t>
+          <t>Fri, 23 Oct 2026 22:09:00 GMT</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxQVFFlUGRwNDZuVldGdVB1UTZtakZuX3dtQjkzUUFhaDFrX0RfZUE4SFoxUmRLMzYzMVNGdDVmWUJyR1N2UVBxTi1zWkhmbWt0eGUzRUxPZW5mN1dQMnZILUhLMWYyRm40dURxbmo1Z2hpYXZBckotZVlGUUt1eFQ4N0IwcnJZOWg2eVdpdDI5eVdCdTlyZ1RBbjlpSjhZSGU2R2hWVmN5b2thZGxzTGtfd2NTQnRFZzkwNFE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMinAFBVV95cUxNZExyeHNLSlFfMllzbWt3cjlLakhlTzhJMThleGp6NmxrendmaWJiYlVEMnViT2tuNnE4TS1hVXpSdUh4SWZwcTdUSzdrOWgtUjdtSzRMUElJMmhEclFraV83cmRoWmN4RGZJaUNkdXlzUG13eHNZT0pKWkFxYUM1Q2lkcHc2amtDZkZZcU96bC00WEVqaFNNMlJ4VWw?oc=5</t>
         </is>
       </c>
     </row>
@@ -747,27 +747,27 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Broker Warns Self-Funded Plans on Rising Costs and PBM Pressures</t>
+          <t>Navigating Pharmacy Compliance and Legislative Impact for Self-Funded Employers</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Insurance brokers are sounding the alarm for self-funded health plans regarding escalating healthcare costs and the urgent need for better plan management. This directly impacts employer health strategies and highlights the growing pressure on pharmacy and medical benefit structures. The report underscores why employers are increasingly seeking transparent, unbundled PBM solutions to control rising spend.</t>
+          <t>Mercer outlines upcoming pharmacy compliance challenges driven by recent legislative changes affecting employer-sponsored health plans. The guidance highlights how shifting regulations impact plan design, cost management, and fiduciary responsibilities for self-funded employers. Self-funded plan sponsors must closely monitor these compliance shifts to adapt their PBM strategies and avoid regulatory pitfalls.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Insurance Business</t>
+          <t>www.mercer.com</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 18:43:55 GMT</t>
+          <t>Fri, 23 Oct 2026 21:08:21 GMT</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiywFBVV95cUxOczExbWJUYlpvWWl5aXY4QVJiaHlFZE1XSDFnOWNfQ0ctRUpJazE4ZEF2UnA0UXRnb0RLcTBKZFpDZGlJNTAyaFlibGNFVWVFb0h5aVFzb3NyNGRlNGZKazBSeTNEcTFUWk9oRXFMbm4zNEphUWU2ZE1iVl9IZVFYYmJ1cDE5M1k1QlZfVF9jM1FDdTZUS1NDY0g4V0xiVGhGZEIybEFVbUMtUTUwTHJVWFVtUVFoTld6bUhiVkFwMGtDd2tHZkFia2xqOA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE5qeFo0X182QVRPOHdlR0t1NHRwVXF1elZlOWRhcUNEdDk4SjZsVWdsRGtEU0Z0R1JqNE1tcFFJa2VmQ2pDaXVISG5rbk9URFViOWdiUk91SC1RM1RwQkRGeGEzZFNuZlE3TC1ZcVNLM1Z2eDVfZVpkeXYwbw?oc=5</t>
         </is>
       </c>
     </row>
@@ -777,27 +777,27 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>AMA Report Highlights Expanding Market Influence of PBMs</t>
+          <t>Employers Health Partners With Archimedes to Cut Pharmacy Costs</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>A new American Medical Association report details the growing market consolidation and influence of pharmacy benefit managers across the US healthcare system. This heightened scrutiny emphasizes the ongoing pressure self-funded employers face regarding PBM transparency, pricing practices, and plan management.</t>
+          <t>Employer coalition Employers Health has selected PBM Archimedes to provide cost-reduction strategies and alternative pharmacy benefit solutions for its members. This move highlights growing demand among employer groups for specialized PBM alternatives aimed at driving down self-funded drug spend. The partnership underscores competitive pressures in the PBM market as coalitions seek greater transparency and savings.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Healthcare Brew</t>
+          <t>Business Wire</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 18:59:52 GMT</t>
+          <t>Fri, 23 Oct 2026 14:00:00 GMT</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxNT0J5QjRDanF1bi1CTjBTMTdyNHRVUDRBcXFHeERxSG1helZWNlAxRDllUVhPN3I4WElUck9EZnJ5eW5ZV0hNTG5nQWtCNmxwVjlON1lQN1ZnNFJDOG16MXFOWVZXd0dqb2o0ZGlOblVTbXNoWUtmcmNlcTd5N0IwN1JldUM1TDdFLWowTUIxTGRGaHBuSGw2Q0ZCQ0pkcEpqX3hkN2FUdlNka0o1TmxYWA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPaXZqS2VhMDdiSVo0dU9tRnVka2poUnVCWWtJa3lfbjNVT2RuSHJwU0NwRTM3am1GRllyRkROTFpQUzFCYktLMVZQSWxmbzJZdWkwRmFTelMtV0tUWndFU0FFSnFJYlo5d29hMHZnYXlWWVdabHpWSXBxNV9pSDdVTHpwZTVsVHNWdGJpQjYzN2liT0F5cTB0dm56ajhYeGZUOGVPNXBudjRzSU05?oc=5</t>
         </is>
       </c>
     </row>
@@ -807,27 +807,27 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>AI Streamlines Specialty Pharmacy Workflows and Prior Authorizations</t>
+          <t>Epic Systems Launches Prescription Marketplace to Enhance Price Transparency</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Artificial intelligence is transforming specialty pharmacy operations by automating complex workflows and prior authorization processes in 2026. For self-funded employers and PBMs, these technological efficiencies can reduce administrative bottlenecks and lower the operational costs associated with high-cost specialty drugs.</t>
+          <t>Epic Systems has introduced a new prescription marketplace aimed at providing greater price transparency and lowering drug costs for patients and healthcare providers. For self-funded employers and PBMs, this technology could disrupt traditional pharmacy benefit navigation by exposing real-time drug pricing at the point of care. The development highlights increasing industry pressure for end-to-end transparency in prescription drug costs.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Pharmacy Times</t>
+          <t>The American Action Forum</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 19:33:29 GMT</t>
+          <t>Fri, 23 Oct 2026 13:57:24 GMT</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxNRldoVW4wZ1FZaDc1UEd0SUVCTUR5N2VkRVJDQ1dybTVWQlBvLVRGTlE3OEh4bDY3cEVYd245OVgzc2VMMW1INmFWS2pSZ19uOWJ1bzRfMjdBbEJOSXBpVGIzeTZxN0xSNlhSTm9temxtWl9iMUhqd1FVRDlQdFA5WG9RZVlEbnZnTkJCb01LUjBKSzVNSVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxOc29CTm5ZU2R4Vkd1cklSb0hsT0hKQ1hMa20wNUl6NFpOcUktdEZKbmxJUGtwVTFHTWJfY1dDWUtkMEFRSmlXbDFHcHZjSS1mSXhDZWZWanJmNEJ4MTBhV3cyVGxWR3o0b190ZmxfaWZkOHJla0djVmRaZmR1NlRINlNab2RubXlCWVdDVUlXMjhhejJtNVd1S3lHUFc2aEdQSlZmWkNEMkI5QXpsNzE4QnFqOFR6M1RuWmpGLXktTVkxcGs?oc=5</t>
         </is>
       </c>
     </row>
@@ -837,27 +837,27 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Job-Based Health Plan Costs Continue Escalating With No Relief in Sight</t>
+          <t>Samsung Bioepis Report Emphasizes Biosimilar Supply Continuity for Payers</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>A new KFF report highlights ongoing, steep increases in employer-sponsored health plan costs, putting intense pressure on self-funded employers. These escalating expenses underscore the urgent need for plan sponsors to adopt aggressive cost-containment strategies, particularly around pharmacy benefits and specialty drug management.</t>
+          <t>Samsung Bioepis released its Q4 2026 market report highlighting the critical role of supply chain reliability in biosimilar adoption. For self-funded employers and PBMs, ensuring consistent supply is essential to capturing projected cost savings from complex biologic alternatives. The report underscores that formulary design must account for both price and manufacturer stability to avoid disruption in patient care.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>KFF Health News</t>
+          <t>BioSpace</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 09:03:03 GMT</t>
+          <t>Fri, 23 Oct 2026 02:38:58 GMT</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxOTll5ai1rdUx3aG5FVEV2OE1QSnhxN0lwcnprODVwSW4zem40SERCMzZiaXE1ZFV4OHNRV0d6RHFkWDhacEgtU29ZWTJsQTRkOUhuNUg2U21UdmJOdnBnNS0xaUtYQnRKdnp4M0pWWEw0Q3owc2plSS1Ka216OEhJSkV3Qmt6SUZnZUpNZ3h2Tm96dUFjMGQzVDVVUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6gFBVV95cUxQS19pN0J0SzBQTlAxRHcxQV9Dc0VQaGpxM3hnNkFzSlVyZS0wT3BSTmFWLTVkZlZxZlJGcE9KblBXeWNzS3VkeVlqbVNqOTZsdlo1VUFsX05vdGxETnVsWVFqMlNEQkNETnpIaEZkNkprNDI1M2w1N1dvbVl6QU81Z1JxQl9fSGdJa29pTFEyLXh6N2NabXVkRXlMM0pBVHN6akJvMUQzWlhPSzJQT3l6bHkwVlVQeXFhTllMeW91TkR6b0xGM3JDNzhoSjg0V2xnQ0Z2T3VReWszMkhGdzdCNTRLOFlqNEpkWVE?oc=5</t>
         </is>
       </c>
     </row>
@@ -867,27 +867,27 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Samsung Bioepis Releases Q4 Biosimilar Market Report Highlighting Adoption Trends</t>
+          <t>Major Companies Pledge Faster Electronic Prior Authorizations</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Samsung Bioepis has published its Q4 Biosimilar Market Report, tracking utilization and market dynamics for key biologic alternatives. The report provides critical insights into biosimilar uptake, which is a major strategy for self-funded employers and PBMs looking to mitigate rising specialty drug costs. Tracking these market shifts helps plan sponsors optimize their formularies to capture meaningful pharmacy savings.</t>
+          <t>Five major healthcare companies have committed to streamlining and accelerating prior authorization processes using electronic standards. This shift aims to reduce administrative friction and care delays, directly impacting specialty drug management and utilization review workflows for employer-sponsored plans.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Drug Store News</t>
+          <t>Healthcare Dive</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 12:52:00 GMT</t>
+          <t>Fri, 23 Oct 2026 15:54:28 GMT</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxQdEktX3Q5Q1NrWTl5YTNsVGQzWXJ4ck45YzRtSms0MUk0aVNRZWx3S1FxWkZ3MUx3SWtnUnd0WjUxU3g1RkdOanNYTU5BaUsycWFFYzQ3NXJaejlnbHI4aHQ1bnFHNlBhRnZ5bEY4a2V4REJHMWZBd0VMQVhDUzkxUmtqam0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNTUxNTklxcEJHcjJFWFFiT3dQMUEyUmtmVEQwQmJMYS1xU2hDdHBjWXBUZHhVR01zWGhOeE1CZFdWdjhIZjJvVmZtSHF2Mms2UkZoNXJXOGVOM3Bzd1JOeklCb0Y0X2VUbkZaa3VyRVY4eVFOcjFKbW1Ma3l5cFkxYjI0VW1fVzJscFRoR0t1QnYxbjNoWEVBcWdCdlB6LWV4Rk4wRk1vN2FxbU45NXFr?oc=5</t>
         </is>
       </c>
     </row>
@@ -897,27 +897,27 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Telehealth Platforms Drive Off-Label GLP-1 Prescriptions for Addiction</t>
+          <t>HRSA Revisits 340B Rebate Model with New Pilot Proposal</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Telehealth providers are increasingly prescribing GLP-1 receptor agonists off-label for substance use disorders and addiction ahead of official FDA approvals. This trend introduces complex utilization management and cost challenges for self-funded employers whose health plans must navigate coverage decisions and prior authorization policies for emerging, high-cost off-label uses.</t>
+          <t>HRSA is exploring a new pilot proposal regarding the 340B rebate model, which could impact drug pricing and distribution dynamics. This regulatory shift is crucial for PBMs and self-funded employers monitoring 340B program integrity and specialty drug cost trends.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>STAT</t>
+          <t>Norton Rose Fulbright</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 08:33:55 GMT</t>
+          <t>Fri, 23 Oct 2026 09:14:53 GMT</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxNc1dVanNlX1U4QVFrSE5JOGxlNDduTVZtOGM4Q2RsemI4RFc4UHhhRklEdXZXbDU5Z0FYQzk3OTBGX0wyeXlyV3h3d0pfWDlMNFprVEE4ajF0c3BfUEV0ZXNRemFpZW9JaVNSYXY5bFVtUTA0UTZTZ09aemVmdk1XXzZ5TVpLX1gyendIVXJxSFU5TW5MWlNOQTdiRjdiVFByMWZ1SGVlZU4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxOdjhwcEVhd2JFWmZpTGlpbTFNZGZWSjJpQy0tb1JhelRrZWZlWWZxeUVkOTNxMmlVTmt1N0Jocm5vWmhBT2hFMWxJNmppQTllcTlPM3JTbWRsR2ZtQk1oZUxNWm5FWHI0ejI3dm9zR1pQc3dJbWJ0SzV5Smhqc1Y5emphTnV6STFpek9tX1VmUFJjcXVUbkc0X0ZoWVpLakx4UU9ORjJid0JJSlpaTHVEWmJ5RXJybkxZX3ZFeWJmQ3prT1JfR0xGSnVB?oc=5</t>
         </is>
       </c>
     </row>
@@ -927,27 +927,27 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Weight Loss Now Drives Majority of GLP-1 Utilization, Research Shows</t>
+          <t>Texas Employers Lose $353M Annually Due to 340B Program Expansion</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Recent research reveals that more patients now take GLP-1 medications for weight loss than for managing other health conditions like type 2 diabetes. This shift highlights the accelerating volume of cosmetic and obesity-related prescriptions driving up pharmacy benefit expenditures. For self-funded employers, this trend underscores the urgent need for strategic benefit design, tight utilization management, and careful formulary oversight to control surging plan costs.</t>
+          <t>A new report reveals that Texas employers absorb $353 million in annual costs as the 340B drug discount program expands with minimal transparency. This financial impact underscores the ongoing cost burden placed on self-funded health plans by complex drug pricing and distribution loopholes. The findings highlight the critical need for employer advocacy and greater transparency in pharmacy benefit operations.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>CBS News</t>
+          <t>The Business Journals</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 21:58:53 GMT</t>
+          <t>Fri, 23 Oct 2026 20:08:00 GMT</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwFBVV95cUxNRWNOc2lwSzR4LThkTHNBdXBRMGVjeGVsekdpbjcyYkVDY3dCTU5fZFNaM2xtRW5WOHpNellOdnhRTE52eE5Kc0MwdDJ5djBuaFdTZDFicm1xNkRTRWFhVWJYTkdocXNZbW1IWFlxUmZvQS1UUThHdERoUno2RS1mUy15NHlocTg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxObWZVa1BVZGdpMVVHUW8tN2c2ZnJONklfdTgxNVZFUUduVDdJNWdjbjZFekRrYmdvYUhsdUFoYWJWd1hYMGNrTmMzZ1ZPUm9mTllDekhycEg1MmJxNDc4Ui1Xc0FUMlFxd2E2VmZNbWNXN3dYUm91Tm5kd3FibGEwV3lDd0ZaVWVsVllWckpkZmd4elN0alRESGY1aDFTdHdHdTRv?oc=5</t>
         </is>
       </c>
     </row>
@@ -957,207 +957,27 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>State Attorneys General Sue Insulin Manufacturers and PBMs Over Pricing Schemes</t>
+          <t>House Panel Targets Major PBMs in Ongoing Drug Pricing Investigation</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Florida and multiple other states have filed lawsuits against major insulin manufacturers and pharmacy benefit managers (PBMs), alleging deceptive pricing schemes that artificially inflate patient costs. This litigation intensifies regulatory scrutiny on PBM pricing practices and rebate structures, directly impacting self-funded employer health plans navigating drug cost transparency.</t>
+          <t>A new congressional investigation has been launched targeting the largest PBMs—CVS Caremark, Express Scripts, and Optum Rx—over their business practices and drug pricing models. This regulatory scrutiny increases pressure on traditional PBM transparency and could accelerate legislative reforms affecting self-funded employer health plans.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Florida Daily</t>
+          <t>Seeking Alpha</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Thu, 22 Oct 2026 10:06:56 GMT</t>
+          <t>Fri, 23 Oct 2026 16:14:33 GMT</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiyAFBVV95cUxOV2tvbXpKb3F2YzVDQ0ZyRVhmUGc1NWtFVTVTcnRIbG9NX2s4c1o5ZVNqQ2dKajZuMHVHVE9IWlVhaWhaaWxsdlRzSElESFpaaDhMbS16d0J6VXVlVUZma3NEQmtfOUZocVlIeU5tQ0ZnaEpJYUMxYk9kbDlUbFNUVGJ5MEFtMWxZVDAwcUJEdDNfWDJzMFhWengyejRzazVHc3Vwa1dTVFNwLXVsVjBVQ1pYVklpdE54NjAyZEREZlBsLWhZVGp3Yg?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>UnitedHealthcare Eliminates 30 Percent of Prior Authorization Requirements</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>UnitedHealthcare announced it is dropping approximately 30 percent of its prior authorization requirements to streamline care delivery and reduce administrative burden. This shift by a major national payer highlights broader industry movement away from heavy utilization management, which self-funded employers and PBMs monitor closely for its impact on patient access and medical versus pharmacy cost trends.</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Medical Economics</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Thu, 22 Oct 2026 21:43:58 GMT</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiygJBVV95cUxQX1JDRlgtMmgyOVZMMURwNkFmTFZfY19lNEZ6Rm5qUEtBLUdWNVZyOTJnSVc4YXFpS2ROZEVTQnk0TVFfY2FzRUhNMHg2bmc0MHZnSUJ6QXlDWjBjeGpkaVBCenY2N0JDOHgwc3hoanVFZFZKS0RKX0VOdEV2RVFaa2dxN1pXakI2UTlnSzJIdkNoUjY4TXdSVW1WSzFodktuSUE5N0ZrR1FlblozekxnaVFwbEduOTRyZkhQX3MxZmZacWc3SnZXMllGWUxjM2Y2WmJQR2U0MzZLTXZfd21MRlpiZW9oWWMzSGc1RnNjd0kxTC1oYTNIaXo1cDJmb25mbWo0SXloQkFZY3Rfc0tkRFpSQmJ5M2NSOTYtT1JEVzRhQnZEMThaaFlQT0U1RGZkakQ2VEtVaTBkTHJIVks3OF9wZUgwVUJPU1E?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>HRSA Reevaluates 340B Rebate Model With New Pilot Proposal</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>The Health Resources and Services Administration is revisiting the 340B drug pricing program with a new rebate model pilot proposal. This regulatory shift could significantly impact drug pricing dynamics, manufacturer restrictions, and pharmacy benefit management for self-funded employer health plans navigating 340B compliance and savings.</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Norton Rose Fulbright</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Thu, 22 Oct 2026 15:54:35 GMT</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxOQWFNQ0lVMXhUeDJIX2kwLThXTHN6RUx1Zm1pNU54enUtXzlFZGhtSFotUzJrTnluSlFUbUZUQkYxZkY0UzVfOHhvcUk4RlZuVU9uVzZzRkRLeTlfa3NWdFJjd0NGVGsyNDNTWGhVN2ItOVFqVnBNTWNQc2dGYkh5SFF5c0dpS0RTWGR0cV9CUTBGVHYzRnZHQkxJQW5vZTM2NW5TdUpjUDJvN3MyWFBneFdPaER5d1dDYmU5RXgwOFNaTUl1V2c?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Employer Health Insurance Costs Projected to Rise 9%</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Employer-sponsored health insurance costs are expected to increase by approximately 9% during open enrollment, placing additional financial strain on self-funded plans. This trend highlights the growing urgency for employers to implement effective cost management strategies, particularly around specialty and pharmacy benefits.</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>NBC Palm Springs</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Thu, 22 Oct 2026 19:25:23 GMT</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi0AFBVV95cUxOa0t5ejFWMVFkMmt5ZHZ2QWFSZkdhR0h2YUZJbHhWb3ZFVF9IdEh3SDlFRHpsV0oyNU11a3k3R29iOWJEaE5oanVvLUZ4ZWJ5YUFydVh3NFQwTmR2WTVERmItWEg2XzJ3akt4bUhacTVvS01iR1JaZEFBTUViMGEzejNscGg1MlkxU3p4eDF3ZFpQcHlqUW0zMVYySzBEYl9CRjJ1bVBWbUREZDBsQkkyWjUwbE9QUjBtVk9DMVVNUXA0WkliTXJiQzBsclNub3Vr?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Family Health Insurance Premiums Exceed $28,000 Amid Rising Costs</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Average family health insurance premiums have surpassed $28,000, driven by a 9% increase in worker contributions. This ongoing surge in healthcare and pharmacy benefit costs places additional financial strain on self-funded employers seeking sustainable cost management strategies.</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Healthcare Finance News</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Thu, 22 Oct 2026 14:48:54 GMT</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxQLUpOZDZMRksyYk9aSUY1OHNhQ0pyUW44Zm14cGhWZmQtbEJCb1M2cnM1dUcwVWE3Tm1wd2NMWkQzNU42TExLODUwTG9zVXdzalFtRTlQUFg1amVma1RNSHFpTnVOZVNIM3BQdmpUbmxTMjNrUGU1YWRNcElKLWtnTGU0bHdhbllqYWV5dmtYem1aNERUSzRSOTN0ZmtkMFZDZEFkZnFR?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Employer Healthcare Costs Surge Near 10% With Rising Employee Burden</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Commercial healthcare costs are projected to spike by nearly 10%, placing increased financial strain on both self-funded employers and their workforce. This acute cost inflation heightens the urgency for plan sponsors to optimize pharmacy benefit management, control specialty spend, and reevaluate benefit designs.</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Barron's</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Thu, 22 Oct 2026 09:00:00 GMT</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxNM0Y3Y2dPRlRva21weS0wVlJ2cVZBdVFiTmNnTnR6bUR4dDQ1LXc2NW5JODQzUFNxXzFsZVNmOW14OEtMd3RGN2M2RW1oUlI3Q0t5c3lCRjhYLWVEZVliYmtqSHFIVTZRZ0xhYVVIUEJ4OTEzaG45dm1ScjVUOFBienM5T3NweVlNS3ZyYzdFSQ?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Illinois Judge Questions Bid to Block State 340B Drug Discount Law</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>An Illinois federal judge is showing skepticism toward a pharmaceutical industry challenge aimed at blocking a state law protecting 340B drug discounts. The outcome could set a precedent for state-level oversight of drug pricing and manufacturer restrictions, impacting overall pharmacy benefit costs and supply chain dynamics for self-funded plans.</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Law360</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Thu, 22 Oct 2026 01:32:16 GMT</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMizwFBVV95cUxQaWZ6VFFiS3Y5RWc0dVBtMDNGcGtCTGxkb3R1TWJ1TWVYcUJkc2ZYMVA0QTB3aWV3RUo2SjV2TllQSTduMnlyNmR5UkVZMDdSY2dqdndwR1pPcVFnWkhsLUFMMnhfMm84Z2pEVkFCazV2Szk2UnRIMVhyMl9PQkdwY1RzVFhOeGRFZU9KclE2aFV2TEhJUENCLS1heUdFS2xBb1hXaEphSmU1T1FIMFctcTdkZWlmNzlNaGZkdl8zNFBIOEF5TzRNeTVTbUtjZU3SAXJBVV95cUxPR1l6bTBqVW5Vc2lRWlFyckhkR2FKSU5PRnV1ek1JNHFaelRQTVc0UlphakdqYzJpeEZQVE9MV1hMdkhPYnd3aVBXek13VlIwdzNOV1Bab0RseHU3UXVoYmRNUlB2N3V0MFVqQmdOelVCd1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxQSkRXTnBka1hlLS1QZUh0UHpoQTVMOVJQX2ZiN2hmQ1B0TWpBMU05NzY3RVVaX0t6V1c1SVRzUS14aHBibFZJcEZuaVl5dWNGaE5rMGVpTzN0SWNHd29uYXBYQVV0M1dnR3FvN0VlZERRM0JLa2E4SXcyanc3WnVObWhPY1hkaThUb0R1NlJ3V0kyM3lSYUVXRTNMQkV3YS1rRzVJWUNJZw?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>